<commit_message>
Fix Adding Test Signal to excel sheet
</commit_message>
<xml_diff>
--- a/Task 2/ECG_Feature_Map.xlsx
+++ b/Task 2/ECG_Feature_Map.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP4"/>
+  <dimension ref="A1:AP3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -884,136 +884,6 @@
       </c>
       <c r="AP3" t="n">
         <v>0.005318054410943369</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Test_Signal</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>7.28448275862069</v>
-      </c>
-      <c r="C4" t="n">
-        <v>1.706003772092075</v>
-      </c>
-      <c r="D4" t="n">
-        <v>7.379310344827586</v>
-      </c>
-      <c r="E4" t="n">
-        <v>3.215413236739008</v>
-      </c>
-      <c r="F4" t="n">
-        <v>12.80811704416673</v>
-      </c>
-      <c r="G4" t="n">
-        <v>3.141997135956129</v>
-      </c>
-      <c r="H4" t="n">
-        <v>1031.212710715128</v>
-      </c>
-      <c r="I4" t="n">
-        <v>1323.203672779076</v>
-      </c>
-      <c r="J4" t="n">
-        <v>2531755113.947025</v>
-      </c>
-      <c r="K4" t="n">
-        <v>515.8957056635929</v>
-      </c>
-      <c r="L4" t="n">
-        <v>1042.068475750417</v>
-      </c>
-      <c r="M4" t="n">
-        <v>1570728837.836962</v>
-      </c>
-      <c r="N4" t="n">
-        <v>207.7760813085587</v>
-      </c>
-      <c r="O4" t="n">
-        <v>580.4515526769527</v>
-      </c>
-      <c r="P4" t="n">
-        <v>972388866.2977121</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>41.35349455037417</v>
-      </c>
-      <c r="R4" t="n">
-        <v>126.3545472139302</v>
-      </c>
-      <c r="S4" t="n">
-        <v>92040943.79161854</v>
-      </c>
-      <c r="T4" t="n">
-        <v>3.116343599963999</v>
-      </c>
-      <c r="U4" t="n">
-        <v>9.657595379937566</v>
-      </c>
-      <c r="V4" t="n">
-        <v>1074740.398431321</v>
-      </c>
-      <c r="W4" t="n">
-        <v>0.003294039229342063</v>
-      </c>
-      <c r="X4" t="n">
-        <v>0.004905922342896265</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>0.004853468746472776</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>0.004837029011112378</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>0.00485524559025388</v>
-      </c>
-      <c r="AB4" t="n">
-        <v>0.004833706764302221</v>
-      </c>
-      <c r="AC4" t="n">
-        <v>0.004858268824553343</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>0.004835541988876719</v>
-      </c>
-      <c r="AE4" t="n">
-        <v>0.004862659643426312</v>
-      </c>
-      <c r="AF4" t="n">
-        <v>0.00483930894022197</v>
-      </c>
-      <c r="AG4" t="n">
-        <v>0.004868581495455734</v>
-      </c>
-      <c r="AH4" t="n">
-        <v>0.004844397802787174</v>
-      </c>
-      <c r="AI4" t="n">
-        <v>0.0048761989347621</v>
-      </c>
-      <c r="AJ4" t="n">
-        <v>0.004850400175150253</v>
-      </c>
-      <c r="AK4" t="n">
-        <v>0.004886166090983041</v>
-      </c>
-      <c r="AL4" t="n">
-        <v>0.004856979853945057</v>
-      </c>
-      <c r="AM4" t="n">
-        <v>0.004897399283754211</v>
-      </c>
-      <c r="AN4" t="n">
-        <v>0.004866261140666215</v>
-      </c>
-      <c r="AO4" t="n">
-        <v>0.004915563972039156</v>
-      </c>
-      <c r="AP4" t="n">
-        <v>0.004876935215506006</v>
       </c>
     </row>
   </sheetData>
@@ -1027,7 +897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1110,31 +980,6 @@
       </c>
       <c r="G3" t="n">
         <v>1.298667195539532</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Test_Signal</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>7.28448275862069</v>
-      </c>
-      <c r="C4" t="n">
-        <v>1.706003772092075</v>
-      </c>
-      <c r="D4" t="n">
-        <v>7.379310344827586</v>
-      </c>
-      <c r="E4" t="n">
-        <v>3.215413236739008</v>
-      </c>
-      <c r="F4" t="n">
-        <v>12.80811704416673</v>
-      </c>
-      <c r="G4" t="n">
-        <v>3.141997135956129</v>
       </c>
     </row>
   </sheetData>
@@ -1148,7 +993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1330,58 +1175,6 @@
       </c>
       <c r="P3" t="n">
         <v>560267.5649041033</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Test_Signal</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1031.212710715128</v>
-      </c>
-      <c r="C4" t="n">
-        <v>1323.203672779076</v>
-      </c>
-      <c r="D4" t="n">
-        <v>2531755113.947025</v>
-      </c>
-      <c r="E4" t="n">
-        <v>515.8957056635929</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1042.068475750417</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1570728837.836962</v>
-      </c>
-      <c r="H4" t="n">
-        <v>207.7760813085587</v>
-      </c>
-      <c r="I4" t="n">
-        <v>580.4515526769527</v>
-      </c>
-      <c r="J4" t="n">
-        <v>972388866.2977121</v>
-      </c>
-      <c r="K4" t="n">
-        <v>41.35349455037417</v>
-      </c>
-      <c r="L4" t="n">
-        <v>126.3545472139302</v>
-      </c>
-      <c r="M4" t="n">
-        <v>92040943.79161854</v>
-      </c>
-      <c r="N4" t="n">
-        <v>3.116343599963999</v>
-      </c>
-      <c r="O4" t="n">
-        <v>9.657595379937566</v>
-      </c>
-      <c r="P4" t="n">
-        <v>1074740.398431321</v>
       </c>
     </row>
   </sheetData>
@@ -1395,7 +1188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:U3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1632,73 +1425,6 @@
       </c>
       <c r="U3" t="n">
         <v>0.005318054410943369</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Test_Signal</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0.003294039229342063</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.004905922342896265</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.004853468746472776</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.004837029011112378</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.00485524559025388</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.004833706764302221</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.004858268824553343</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.004835541988876719</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.004862659643426312</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.00483930894022197</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.004868581495455734</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.004844397802787174</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0.0048761989347621</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0.004850400175150253</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0.004886166090983041</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0.004856979853945057</v>
-      </c>
-      <c r="R4" t="n">
-        <v>0.004897399283754211</v>
-      </c>
-      <c r="S4" t="n">
-        <v>0.004866261140666215</v>
-      </c>
-      <c r="T4" t="n">
-        <v>0.004915563972039156</v>
-      </c>
-      <c r="U4" t="n">
-        <v>0.004876935215506006</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
change sampling rate with normalized features
</commit_message>
<xml_diff>
--- a/Task 2/ECG_Feature_Map.xlsx
+++ b/Task 2/ECG_Feature_Map.xlsx
@@ -633,127 +633,127 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7.28448275862069</v>
+        <v>12.90222222222222</v>
       </c>
       <c r="C2" t="n">
-        <v>1.706003772092075</v>
+        <v>7.070391750544863</v>
       </c>
       <c r="D2" t="n">
-        <v>7.379310344827586</v>
+        <v>12.14222222222222</v>
       </c>
       <c r="E2" t="n">
-        <v>3.215413236739008</v>
+        <v>6.784770163597254</v>
       </c>
       <c r="F2" t="n">
-        <v>12.80811704416673</v>
+        <v>3.331408705329584</v>
       </c>
       <c r="G2" t="n">
-        <v>3.141997135956129</v>
+        <v>7.275447915055158</v>
       </c>
       <c r="H2" t="n">
-        <v>1031.212710715128</v>
+        <v>934.6396744397169</v>
       </c>
       <c r="I2" t="n">
-        <v>1323.203672779076</v>
+        <v>1200.651186954293</v>
       </c>
       <c r="J2" t="n">
-        <v>2531755113.947025</v>
+        <v>2084501830.818344</v>
       </c>
       <c r="K2" t="n">
-        <v>515.8957056635929</v>
+        <v>517.7336695298392</v>
       </c>
       <c r="L2" t="n">
-        <v>1042.068475750417</v>
+        <v>1046.519376255087</v>
       </c>
       <c r="M2" t="n">
-        <v>1570728837.836962</v>
+        <v>1584171996.317703</v>
       </c>
       <c r="N2" t="n">
-        <v>207.7760813085587</v>
+        <v>225.1470932343341</v>
       </c>
       <c r="O2" t="n">
-        <v>580.4515526769527</v>
+        <v>680.8324096253896</v>
       </c>
       <c r="P2" t="n">
-        <v>972388866.2977121</v>
+        <v>1338078347.1281</v>
       </c>
       <c r="Q2" t="n">
-        <v>41.35349455037417</v>
+        <v>60.50425213733803</v>
       </c>
       <c r="R2" t="n">
-        <v>126.3545472139302</v>
+        <v>214.6277029303527</v>
       </c>
       <c r="S2" t="n">
-        <v>92040943.79161854</v>
+        <v>265565018.2470056</v>
       </c>
       <c r="T2" t="n">
-        <v>3.116343599963999</v>
+        <v>6.667193842428753</v>
       </c>
       <c r="U2" t="n">
-        <v>9.657595379937566</v>
+        <v>23.08270275014829</v>
       </c>
       <c r="V2" t="n">
-        <v>1074740.398431321</v>
+        <v>6139583.068739802</v>
       </c>
       <c r="W2" t="n">
-        <v>17012655.12929675</v>
+        <v>0.00329403922934207</v>
       </c>
       <c r="X2" t="n">
-        <v>25337513.94559935</v>
+        <v>0.004749936946592341</v>
       </c>
       <c r="Y2" t="n">
-        <v>25066607.95932712</v>
+        <v>0.004719038117735614</v>
       </c>
       <c r="Z2" t="n">
-        <v>24981702.00386302</v>
+        <v>0.004728374218786425</v>
       </c>
       <c r="AA2" t="n">
-        <v>25075784.7870337</v>
+        <v>0.004719362166154055</v>
       </c>
       <c r="AB2" t="n">
-        <v>24964543.66563438</v>
+        <v>0.004727065673040516</v>
       </c>
       <c r="AC2" t="n">
-        <v>25091398.82163708</v>
+        <v>0.004719906358117905</v>
       </c>
       <c r="AD2" t="n">
-        <v>24974022.0113968</v>
+        <v>0.004727233011278142</v>
       </c>
       <c r="AE2" t="n">
-        <v>25114075.99152501</v>
+        <v>0.004720678380960819</v>
       </c>
       <c r="AF2" t="n">
-        <v>24993477.10578498</v>
+        <v>0.004727890801703888</v>
       </c>
       <c r="AG2" t="n">
-        <v>25144660.4561561</v>
+        <v>0.004721688161243556</v>
       </c>
       <c r="AH2" t="n">
-        <v>25019759.4472493</v>
+        <v>0.004728850901437599</v>
       </c>
       <c r="AI2" t="n">
-        <v>25184002.08473565</v>
+        <v>0.004722947026370737</v>
       </c>
       <c r="AJ2" t="n">
-        <v>25050759.77355421</v>
+        <v>0.004730045760717614</v>
       </c>
       <c r="AK2" t="n">
-        <v>25235479.24684606</v>
+        <v>0.004724482926141433</v>
       </c>
       <c r="AL2" t="n">
-        <v>25084741.70224537</v>
+        <v>0.004731441528314515</v>
       </c>
       <c r="AM2" t="n">
-        <v>25293495.08130071</v>
+        <v>0.004726273193273788</v>
       </c>
       <c r="AN2" t="n">
-        <v>25132676.5685751</v>
+        <v>0.004733090946691938</v>
       </c>
       <c r="AO2" t="n">
-        <v>25387309.86485605</v>
+        <v>0.004728492979003365</v>
       </c>
       <c r="AP2" t="n">
-        <v>25187804.73840868</v>
+        <v>0.004734953406203932</v>
       </c>
     </row>
     <row r="3">
@@ -763,127 +763,127 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7.067669172932331</v>
+        <v>8.290123456790123</v>
       </c>
       <c r="C3" t="n">
-        <v>0.6276281730739611</v>
+        <v>5.532934053828734</v>
       </c>
       <c r="D3" t="n">
-        <v>6.984962406015038</v>
+        <v>8.438271604938272</v>
       </c>
       <c r="E3" t="n">
-        <v>1.00363971013488</v>
+        <v>4.924041998728596</v>
       </c>
       <c r="F3" t="n">
-        <v>-5.398425951678979</v>
+        <v>-7.354998402851163</v>
       </c>
       <c r="G3" t="n">
-        <v>1.298667195539532</v>
+        <v>2.891657360811066</v>
       </c>
       <c r="H3" t="n">
-        <v>606.1431668494508</v>
+        <v>604.5821272263487</v>
       </c>
       <c r="I3" t="n">
-        <v>784.1948388763603</v>
+        <v>780.8938728493939</v>
       </c>
       <c r="J3" t="n">
-        <v>889234871.6767075</v>
+        <v>881765226.632076</v>
       </c>
       <c r="K3" t="n">
-        <v>371.447413834591</v>
+        <v>372.7813106039199</v>
       </c>
       <c r="L3" t="n">
-        <v>746.6198155508055</v>
+        <v>750.9423203341649</v>
       </c>
       <c r="M3" t="n">
-        <v>806799804.4576473</v>
+        <v>816167004.876194</v>
       </c>
       <c r="N3" t="n">
-        <v>165.5753551333461</v>
+        <v>181.68636368164</v>
       </c>
       <c r="O3" t="n">
-        <v>436.9476227383831</v>
+        <v>499.3838888145954</v>
       </c>
       <c r="P3" t="n">
-        <v>551005606.8698217</v>
+        <v>719741466.3429611</v>
       </c>
       <c r="Q3" t="n">
-        <v>34.31669556587083</v>
+        <v>49.64595776882005</v>
       </c>
       <c r="R3" t="n">
-        <v>94.35599094623329</v>
+        <v>153.4161094240039</v>
       </c>
       <c r="S3" t="n">
-        <v>51326106.45327463</v>
+        <v>135687961.8067113</v>
       </c>
       <c r="T3" t="n">
-        <v>2.526767447217294</v>
+        <v>4.620747572021741</v>
       </c>
       <c r="U3" t="n">
-        <v>6.972924301393539</v>
+        <v>14.70704859783348</v>
       </c>
       <c r="V3" t="n">
-        <v>560267.5649041033</v>
+        <v>2492393.541350836</v>
       </c>
       <c r="W3" t="n">
-        <v>7537118.359433323</v>
+        <v>0.003294039229342067</v>
       </c>
       <c r="X3" t="n">
-        <v>12265653.65782702</v>
+        <v>0.005115398122532075</v>
       </c>
       <c r="Y3" t="n">
-        <v>11011882.84276245</v>
+        <v>0.00483648952398239</v>
       </c>
       <c r="Z3" t="n">
-        <v>12139662.96994122</v>
+        <v>0.00505145576096159</v>
       </c>
       <c r="AA3" t="n">
-        <v>11011864.71816594</v>
+        <v>0.00483651599497854</v>
       </c>
       <c r="AB3" t="n">
-        <v>12131845.55002127</v>
+        <v>0.005046704855212978</v>
       </c>
       <c r="AC3" t="n">
-        <v>11011799.71766649</v>
+        <v>0.004836564178382793</v>
       </c>
       <c r="AD3" t="n">
-        <v>12132375.2228994</v>
+        <v>0.005045870051113368</v>
       </c>
       <c r="AE3" t="n">
-        <v>11011734.22382049</v>
+        <v>0.004836642622490523</v>
       </c>
       <c r="AF3" t="n">
-        <v>12135600.35633122</v>
+        <v>0.005046082983115644</v>
       </c>
       <c r="AG3" t="n">
-        <v>11011567.75908244</v>
+        <v>0.004836761695586599</v>
       </c>
       <c r="AH3" t="n">
-        <v>12140227.48193748</v>
+        <v>0.005046811815490196</v>
       </c>
       <c r="AI3" t="n">
-        <v>11011387.19423446</v>
+        <v>0.004836935494018355</v>
       </c>
       <c r="AJ3" t="n">
-        <v>12146297.27176641</v>
+        <v>0.005047927435637841</v>
       </c>
       <c r="AK3" t="n">
-        <v>11011157.57001714</v>
+        <v>0.004837182459391151</v>
       </c>
       <c r="AL3" t="n">
-        <v>12152617.88236405</v>
+        <v>0.005049378219682934</v>
       </c>
       <c r="AM3" t="n">
-        <v>11011142.97746135</v>
+        <v>0.004837525719882543</v>
       </c>
       <c r="AN3" t="n">
-        <v>12158627.53702618</v>
+        <v>0.005051162183337258</v>
       </c>
       <c r="AO3" t="n">
-        <v>11008888.84963115</v>
+        <v>0.004837924093448659</v>
       </c>
       <c r="AP3" t="n">
-        <v>12168284.20868341</v>
+        <v>0.005053383494862944</v>
       </c>
     </row>
   </sheetData>
@@ -939,22 +939,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7.28448275862069</v>
+        <v>12.90222222222222</v>
       </c>
       <c r="C2" t="n">
-        <v>1.706003772092075</v>
+        <v>7.070391750544863</v>
       </c>
       <c r="D2" t="n">
-        <v>7.379310344827586</v>
+        <v>12.14222222222222</v>
       </c>
       <c r="E2" t="n">
-        <v>3.215413236739008</v>
+        <v>6.784770163597254</v>
       </c>
       <c r="F2" t="n">
-        <v>12.80811704416673</v>
+        <v>3.331408705329584</v>
       </c>
       <c r="G2" t="n">
-        <v>3.141997135956129</v>
+        <v>7.275447915055158</v>
       </c>
     </row>
     <row r="3">
@@ -964,22 +964,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7.067669172932331</v>
+        <v>8.290123456790123</v>
       </c>
       <c r="C3" t="n">
-        <v>0.6276281730739611</v>
+        <v>5.532934053828734</v>
       </c>
       <c r="D3" t="n">
-        <v>6.984962406015038</v>
+        <v>8.438271604938272</v>
       </c>
       <c r="E3" t="n">
-        <v>1.00363971013488</v>
+        <v>4.924041998728596</v>
       </c>
       <c r="F3" t="n">
-        <v>-5.398425951678979</v>
+        <v>-7.354998402851163</v>
       </c>
       <c r="G3" t="n">
-        <v>1.298667195539532</v>
+        <v>2.891657360811066</v>
       </c>
     </row>
   </sheetData>
@@ -1080,49 +1080,49 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1031.212710715128</v>
+        <v>934.6396744397169</v>
       </c>
       <c r="C2" t="n">
-        <v>1323.203672779076</v>
+        <v>1200.651186954293</v>
       </c>
       <c r="D2" t="n">
-        <v>2531755113.947025</v>
+        <v>2084501830.818344</v>
       </c>
       <c r="E2" t="n">
-        <v>515.8957056635929</v>
+        <v>517.7336695298392</v>
       </c>
       <c r="F2" t="n">
-        <v>1042.068475750417</v>
+        <v>1046.519376255087</v>
       </c>
       <c r="G2" t="n">
-        <v>1570728837.836962</v>
+        <v>1584171996.317703</v>
       </c>
       <c r="H2" t="n">
-        <v>207.7760813085587</v>
+        <v>225.1470932343341</v>
       </c>
       <c r="I2" t="n">
-        <v>580.4515526769527</v>
+        <v>680.8324096253896</v>
       </c>
       <c r="J2" t="n">
-        <v>972388866.2977121</v>
+        <v>1338078347.1281</v>
       </c>
       <c r="K2" t="n">
-        <v>41.35349455037417</v>
+        <v>60.50425213733803</v>
       </c>
       <c r="L2" t="n">
-        <v>126.3545472139302</v>
+        <v>214.6277029303527</v>
       </c>
       <c r="M2" t="n">
-        <v>92040943.79161854</v>
+        <v>265565018.2470056</v>
       </c>
       <c r="N2" t="n">
-        <v>3.116343599963999</v>
+        <v>6.667193842428753</v>
       </c>
       <c r="O2" t="n">
-        <v>9.657595379937566</v>
+        <v>23.08270275014829</v>
       </c>
       <c r="P2" t="n">
-        <v>1074740.398431321</v>
+        <v>6139583.068739802</v>
       </c>
     </row>
     <row r="3">
@@ -1132,49 +1132,49 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>606.1431668494508</v>
+        <v>604.5821272263487</v>
       </c>
       <c r="C3" t="n">
-        <v>784.1948388763603</v>
+        <v>780.8938728493939</v>
       </c>
       <c r="D3" t="n">
-        <v>889234871.6767075</v>
+        <v>881765226.632076</v>
       </c>
       <c r="E3" t="n">
-        <v>371.447413834591</v>
+        <v>372.7813106039199</v>
       </c>
       <c r="F3" t="n">
-        <v>746.6198155508055</v>
+        <v>750.9423203341649</v>
       </c>
       <c r="G3" t="n">
-        <v>806799804.4576473</v>
+        <v>816167004.876194</v>
       </c>
       <c r="H3" t="n">
-        <v>165.5753551333461</v>
+        <v>181.68636368164</v>
       </c>
       <c r="I3" t="n">
-        <v>436.9476227383831</v>
+        <v>499.3838888145954</v>
       </c>
       <c r="J3" t="n">
-        <v>551005606.8698217</v>
+        <v>719741466.3429611</v>
       </c>
       <c r="K3" t="n">
-        <v>34.31669556587083</v>
+        <v>49.64595776882005</v>
       </c>
       <c r="L3" t="n">
-        <v>94.35599094623329</v>
+        <v>153.4161094240039</v>
       </c>
       <c r="M3" t="n">
-        <v>51326106.45327463</v>
+        <v>135687961.8067113</v>
       </c>
       <c r="N3" t="n">
-        <v>2.526767447217294</v>
+        <v>4.620747572021741</v>
       </c>
       <c r="O3" t="n">
-        <v>6.972924301393539</v>
+        <v>14.70704859783348</v>
       </c>
       <c r="P3" t="n">
-        <v>560267.5649041033</v>
+        <v>2492393.541350836</v>
       </c>
     </row>
   </sheetData>
@@ -1300,64 +1300,64 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>17012655.12929675</v>
+        <v>0.00329403922934207</v>
       </c>
       <c r="C2" t="n">
-        <v>25337513.94559935</v>
+        <v>0.004749936946592341</v>
       </c>
       <c r="D2" t="n">
-        <v>25066607.95932712</v>
+        <v>0.004719038117735614</v>
       </c>
       <c r="E2" t="n">
-        <v>24981702.00386302</v>
+        <v>0.004728374218786425</v>
       </c>
       <c r="F2" t="n">
-        <v>25075784.7870337</v>
+        <v>0.004719362166154055</v>
       </c>
       <c r="G2" t="n">
-        <v>24964543.66563438</v>
+        <v>0.004727065673040516</v>
       </c>
       <c r="H2" t="n">
-        <v>25091398.82163708</v>
+        <v>0.004719906358117905</v>
       </c>
       <c r="I2" t="n">
-        <v>24974022.0113968</v>
+        <v>0.004727233011278142</v>
       </c>
       <c r="J2" t="n">
-        <v>25114075.99152501</v>
+        <v>0.004720678380960819</v>
       </c>
       <c r="K2" t="n">
-        <v>24993477.10578498</v>
+        <v>0.004727890801703888</v>
       </c>
       <c r="L2" t="n">
-        <v>25144660.4561561</v>
+        <v>0.004721688161243556</v>
       </c>
       <c r="M2" t="n">
-        <v>25019759.4472493</v>
+        <v>0.004728850901437599</v>
       </c>
       <c r="N2" t="n">
-        <v>25184002.08473565</v>
+        <v>0.004722947026370737</v>
       </c>
       <c r="O2" t="n">
-        <v>25050759.77355421</v>
+        <v>0.004730045760717614</v>
       </c>
       <c r="P2" t="n">
-        <v>25235479.24684606</v>
+        <v>0.004724482926141433</v>
       </c>
       <c r="Q2" t="n">
-        <v>25084741.70224537</v>
+        <v>0.004731441528314515</v>
       </c>
       <c r="R2" t="n">
-        <v>25293495.08130071</v>
+        <v>0.004726273193273788</v>
       </c>
       <c r="S2" t="n">
-        <v>25132676.5685751</v>
+        <v>0.004733090946691938</v>
       </c>
       <c r="T2" t="n">
-        <v>25387309.86485605</v>
+        <v>0.004728492979003365</v>
       </c>
       <c r="U2" t="n">
-        <v>25187804.73840868</v>
+        <v>0.004734953406203932</v>
       </c>
     </row>
     <row r="3">
@@ -1367,64 +1367,64 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7537118.359433323</v>
+        <v>0.003294039229342067</v>
       </c>
       <c r="C3" t="n">
-        <v>12265653.65782702</v>
+        <v>0.005115398122532075</v>
       </c>
       <c r="D3" t="n">
-        <v>11011882.84276245</v>
+        <v>0.00483648952398239</v>
       </c>
       <c r="E3" t="n">
-        <v>12139662.96994122</v>
+        <v>0.00505145576096159</v>
       </c>
       <c r="F3" t="n">
-        <v>11011864.71816594</v>
+        <v>0.00483651599497854</v>
       </c>
       <c r="G3" t="n">
-        <v>12131845.55002127</v>
+        <v>0.005046704855212978</v>
       </c>
       <c r="H3" t="n">
-        <v>11011799.71766649</v>
+        <v>0.004836564178382793</v>
       </c>
       <c r="I3" t="n">
-        <v>12132375.2228994</v>
+        <v>0.005045870051113368</v>
       </c>
       <c r="J3" t="n">
-        <v>11011734.22382049</v>
+        <v>0.004836642622490523</v>
       </c>
       <c r="K3" t="n">
-        <v>12135600.35633122</v>
+        <v>0.005046082983115644</v>
       </c>
       <c r="L3" t="n">
-        <v>11011567.75908244</v>
+        <v>0.004836761695586599</v>
       </c>
       <c r="M3" t="n">
-        <v>12140227.48193748</v>
+        <v>0.005046811815490196</v>
       </c>
       <c r="N3" t="n">
-        <v>11011387.19423446</v>
+        <v>0.004836935494018355</v>
       </c>
       <c r="O3" t="n">
-        <v>12146297.27176641</v>
+        <v>0.005047927435637841</v>
       </c>
       <c r="P3" t="n">
-        <v>11011157.57001714</v>
+        <v>0.004837182459391151</v>
       </c>
       <c r="Q3" t="n">
-        <v>12152617.88236405</v>
+        <v>0.005049378219682934</v>
       </c>
       <c r="R3" t="n">
-        <v>11011142.97746135</v>
+        <v>0.004837525719882543</v>
       </c>
       <c r="S3" t="n">
-        <v>12158627.53702618</v>
+        <v>0.005051162183337258</v>
       </c>
       <c r="T3" t="n">
-        <v>11008888.84963115</v>
+        <v>0.004837924093448659</v>
       </c>
       <c r="U3" t="n">
-        <v>12168284.20868341</v>
+        <v>0.005053383494862944</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
change wavlet coefficients to 3 instead of 4
</commit_message>
<xml_diff>
--- a/Task 2/ECG_Feature_Map.xlsx
+++ b/Task 2/ECG_Feature_Map.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP3"/>
+  <dimension ref="A1:AM3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,175 +452,160 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>DWT_cA4_mean_abs</t>
+          <t>DWT_A3_mean_abs</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>DWT_cA4_std</t>
+          <t>DWT_A3_std</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>DWT_cA4_energy</t>
+          <t>DWT_A3_energy</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>DWT_cD4_mean_abs</t>
+          <t>DWT_D3_mean_abs</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>DWT_cD4_std</t>
+          <t>DWT_D3_std</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>DWT_cD4_energy</t>
+          <t>DWT_D3_energy</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>DWT_cD3_mean_abs</t>
+          <t>DWT_D2_mean_abs</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>DWT_cD3_std</t>
+          <t>DWT_D2_std</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>DWT_cD3_energy</t>
+          <t>DWT_D2_energy</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>DWT_cD2_mean_abs</t>
+          <t>DWT_D1_mean_abs</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>DWT_cD2_std</t>
+          <t>DWT_D1_std</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>DWT_cD2_energy</t>
+          <t>DWT_D1_energy</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>DWT_cD1_mean_abs</t>
+          <t>AC_DCT_0</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>DWT_cD1_std</t>
+          <t>AC_DCT_1</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>DWT_cD1_energy</t>
+          <t>AC_DCT_2</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>AC_DCT_0</t>
+          <t>AC_DCT_3</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>AC_DCT_1</t>
+          <t>AC_DCT_4</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
         <is>
-          <t>AC_DCT_2</t>
+          <t>AC_DCT_5</t>
         </is>
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>AC_DCT_3</t>
+          <t>AC_DCT_6</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
         <is>
-          <t>AC_DCT_4</t>
+          <t>AC_DCT_7</t>
         </is>
       </c>
       <c r="AB1" t="inlineStr">
         <is>
-          <t>AC_DCT_5</t>
+          <t>AC_DCT_8</t>
         </is>
       </c>
       <c r="AC1" t="inlineStr">
         <is>
-          <t>AC_DCT_6</t>
+          <t>AC_DCT_9</t>
         </is>
       </c>
       <c r="AD1" t="inlineStr">
         <is>
-          <t>AC_DCT_7</t>
+          <t>AC_DCT_10</t>
         </is>
       </c>
       <c r="AE1" t="inlineStr">
         <is>
-          <t>AC_DCT_8</t>
+          <t>AC_DCT_11</t>
         </is>
       </c>
       <c r="AF1" t="inlineStr">
         <is>
-          <t>AC_DCT_9</t>
+          <t>AC_DCT_12</t>
         </is>
       </c>
       <c r="AG1" t="inlineStr">
         <is>
-          <t>AC_DCT_10</t>
+          <t>AC_DCT_13</t>
         </is>
       </c>
       <c r="AH1" t="inlineStr">
         <is>
-          <t>AC_DCT_11</t>
+          <t>AC_DCT_14</t>
         </is>
       </c>
       <c r="AI1" t="inlineStr">
         <is>
-          <t>AC_DCT_12</t>
+          <t>AC_DCT_15</t>
         </is>
       </c>
       <c r="AJ1" t="inlineStr">
         <is>
-          <t>AC_DCT_13</t>
+          <t>AC_DCT_16</t>
         </is>
       </c>
       <c r="AK1" t="inlineStr">
         <is>
-          <t>AC_DCT_14</t>
+          <t>AC_DCT_17</t>
         </is>
       </c>
       <c r="AL1" t="inlineStr">
         <is>
-          <t>AC_DCT_15</t>
+          <t>AC_DCT_18</t>
         </is>
       </c>
       <c r="AM1" t="inlineStr">
-        <is>
-          <t>AC_DCT_16</t>
-        </is>
-      </c>
-      <c r="AN1" t="inlineStr">
-        <is>
-          <t>AC_DCT_17</t>
-        </is>
-      </c>
-      <c r="AO1" t="inlineStr">
-        <is>
-          <t>AC_DCT_18</t>
-        </is>
-      </c>
-      <c r="AP1" t="inlineStr">
         <is>
           <t>AC_DCT_19</t>
         </is>
@@ -651,108 +636,99 @@
         <v>7.275447915055158</v>
       </c>
       <c r="H2" t="n">
-        <v>934.6396744397169</v>
+        <v>714.3413889371479</v>
       </c>
       <c r="I2" t="n">
-        <v>1200.651186954293</v>
+        <v>1127.203160402164</v>
       </c>
       <c r="J2" t="n">
-        <v>2084501830.818344</v>
+        <v>3666914081.467175</v>
       </c>
       <c r="K2" t="n">
-        <v>517.7336695298392</v>
+        <v>225.1470932343341</v>
       </c>
       <c r="L2" t="n">
-        <v>1046.519376255087</v>
+        <v>680.8324096253896</v>
       </c>
       <c r="M2" t="n">
-        <v>1584171996.317703</v>
+        <v>1338078347.1281</v>
       </c>
       <c r="N2" t="n">
-        <v>225.1470932343341</v>
+        <v>60.50425213733803</v>
       </c>
       <c r="O2" t="n">
-        <v>680.8324096253896</v>
+        <v>214.6277029303527</v>
       </c>
       <c r="P2" t="n">
-        <v>1338078347.1281</v>
+        <v>265565018.2470056</v>
       </c>
       <c r="Q2" t="n">
-        <v>60.50425213733803</v>
+        <v>6.667193842428753</v>
       </c>
       <c r="R2" t="n">
-        <v>214.6277029303527</v>
+        <v>23.08270275014829</v>
       </c>
       <c r="S2" t="n">
-        <v>265565018.2470056</v>
+        <v>6139583.068739802</v>
       </c>
       <c r="T2" t="n">
-        <v>6.667193842428753</v>
+        <v>0.00329403922934207</v>
       </c>
       <c r="U2" t="n">
-        <v>23.08270275014829</v>
+        <v>0.004749936946592341</v>
       </c>
       <c r="V2" t="n">
-        <v>6139583.068739802</v>
+        <v>0.004719038117735614</v>
       </c>
       <c r="W2" t="n">
-        <v>0.00329403922934207</v>
+        <v>0.004728374218786425</v>
       </c>
       <c r="X2" t="n">
-        <v>0.004749936946592341</v>
+        <v>0.004719362166154055</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.004719038117735614</v>
+        <v>0.004727065673040516</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.004728374218786425</v>
+        <v>0.004719906358117905</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.004719362166154055</v>
+        <v>0.004727233011278142</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.004727065673040516</v>
+        <v>0.004720678380960819</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.004719906358117905</v>
+        <v>0.004727890801703888</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.004727233011278142</v>
+        <v>0.004721688161243556</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.004720678380960819</v>
+        <v>0.004728850901437599</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.004727890801703888</v>
+        <v>0.004722947026370737</v>
       </c>
       <c r="AG2" t="n">
-        <v>0.004721688161243556</v>
+        <v>0.004730045760717614</v>
       </c>
       <c r="AH2" t="n">
-        <v>0.004728850901437599</v>
+        <v>0.004724482926141433</v>
       </c>
       <c r="AI2" t="n">
-        <v>0.004722947026370737</v>
+        <v>0.004731441528314515</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0.004730045760717614</v>
+        <v>0.004726273193273788</v>
       </c>
       <c r="AK2" t="n">
-        <v>0.004724482926141433</v>
+        <v>0.004733090946691938</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.004731441528314515</v>
+        <v>0.004728492979003365</v>
       </c>
       <c r="AM2" t="n">
-        <v>0.004726273193273788</v>
-      </c>
-      <c r="AN2" t="n">
-        <v>0.004733090946691938</v>
-      </c>
-      <c r="AO2" t="n">
-        <v>0.004728492979003365</v>
-      </c>
-      <c r="AP2" t="n">
         <v>0.004734953406203932</v>
       </c>
     </row>
@@ -781,108 +757,99 @@
         <v>2.891657360811066</v>
       </c>
       <c r="H3" t="n">
-        <v>604.5821272263487</v>
+        <v>481.5656708036506</v>
       </c>
       <c r="I3" t="n">
-        <v>780.8938728493939</v>
+        <v>764.7066101312035</v>
       </c>
       <c r="J3" t="n">
-        <v>881765226.632076</v>
+        <v>1687667188.817399</v>
       </c>
       <c r="K3" t="n">
-        <v>372.7813106039199</v>
+        <v>181.68636368164</v>
       </c>
       <c r="L3" t="n">
-        <v>750.9423203341649</v>
+        <v>499.3838888145954</v>
       </c>
       <c r="M3" t="n">
-        <v>816167004.876194</v>
+        <v>719741466.3429611</v>
       </c>
       <c r="N3" t="n">
-        <v>181.68636368164</v>
+        <v>49.64595776882005</v>
       </c>
       <c r="O3" t="n">
-        <v>499.3838888145954</v>
+        <v>153.4161094240039</v>
       </c>
       <c r="P3" t="n">
-        <v>719741466.3429611</v>
+        <v>135687961.8067113</v>
       </c>
       <c r="Q3" t="n">
-        <v>49.64595776882005</v>
+        <v>4.620747572021741</v>
       </c>
       <c r="R3" t="n">
-        <v>153.4161094240039</v>
+        <v>14.70704859783348</v>
       </c>
       <c r="S3" t="n">
-        <v>135687961.8067113</v>
+        <v>2492393.541350836</v>
       </c>
       <c r="T3" t="n">
-        <v>4.620747572021741</v>
+        <v>0.003294039229342067</v>
       </c>
       <c r="U3" t="n">
-        <v>14.70704859783348</v>
+        <v>0.005115398122532075</v>
       </c>
       <c r="V3" t="n">
-        <v>2492393.541350836</v>
+        <v>0.00483648952398239</v>
       </c>
       <c r="W3" t="n">
-        <v>0.003294039229342067</v>
+        <v>0.00505145576096159</v>
       </c>
       <c r="X3" t="n">
-        <v>0.005115398122532075</v>
+        <v>0.00483651599497854</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.00483648952398239</v>
+        <v>0.005046704855212978</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.00505145576096159</v>
+        <v>0.004836564178382793</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.00483651599497854</v>
+        <v>0.005045870051113368</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.005046704855212978</v>
+        <v>0.004836642622490523</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.004836564178382793</v>
+        <v>0.005046082983115644</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.005045870051113368</v>
+        <v>0.004836761695586599</v>
       </c>
       <c r="AE3" t="n">
-        <v>0.004836642622490523</v>
+        <v>0.005046811815490196</v>
       </c>
       <c r="AF3" t="n">
-        <v>0.005046082983115644</v>
+        <v>0.004836935494018355</v>
       </c>
       <c r="AG3" t="n">
-        <v>0.004836761695586599</v>
+        <v>0.005047927435637841</v>
       </c>
       <c r="AH3" t="n">
-        <v>0.005046811815490196</v>
+        <v>0.004837182459391151</v>
       </c>
       <c r="AI3" t="n">
-        <v>0.004836935494018355</v>
+        <v>0.005049378219682934</v>
       </c>
       <c r="AJ3" t="n">
-        <v>0.005047927435637841</v>
+        <v>0.004837525719882543</v>
       </c>
       <c r="AK3" t="n">
-        <v>0.004837182459391151</v>
+        <v>0.005051162183337258</v>
       </c>
       <c r="AL3" t="n">
-        <v>0.005049378219682934</v>
+        <v>0.004837924093448659</v>
       </c>
       <c r="AM3" t="n">
-        <v>0.004837525719882543</v>
-      </c>
-      <c r="AN3" t="n">
-        <v>0.005051162183337258</v>
-      </c>
-      <c r="AO3" t="n">
-        <v>0.004837924093448659</v>
-      </c>
-      <c r="AP3" t="n">
         <v>0.005053383494862944</v>
       </c>
     </row>
@@ -993,83 +960,68 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
-          <t>DWT_cA4_mean_abs</t>
+          <t>DWT_A3_mean_abs</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>DWT_cA4_std</t>
+          <t>DWT_A3_std</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>DWT_cA4_energy</t>
+          <t>DWT_A3_energy</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>DWT_cD4_mean_abs</t>
+          <t>DWT_D3_mean_abs</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>DWT_cD4_std</t>
+          <t>DWT_D3_std</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>DWT_cD4_energy</t>
+          <t>DWT_D3_energy</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>DWT_cD3_mean_abs</t>
+          <t>DWT_D2_mean_abs</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>DWT_cD3_std</t>
+          <t>DWT_D2_std</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>DWT_cD3_energy</t>
+          <t>DWT_D2_energy</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>DWT_cD2_mean_abs</t>
+          <t>DWT_D1_mean_abs</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>DWT_cD2_std</t>
+          <t>DWT_D1_std</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>DWT_cD2_energy</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>DWT_cD1_mean_abs</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>DWT_cD1_std</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>DWT_cD1_energy</t>
+          <t>DWT_D1_energy</t>
         </is>
       </c>
     </row>
@@ -1080,48 +1032,39 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>934.6396744397169</v>
+        <v>714.3413889371479</v>
       </c>
       <c r="C2" t="n">
-        <v>1200.651186954293</v>
+        <v>1127.203160402164</v>
       </c>
       <c r="D2" t="n">
-        <v>2084501830.818344</v>
+        <v>3666914081.467175</v>
       </c>
       <c r="E2" t="n">
-        <v>517.7336695298392</v>
+        <v>225.1470932343341</v>
       </c>
       <c r="F2" t="n">
-        <v>1046.519376255087</v>
+        <v>680.8324096253896</v>
       </c>
       <c r="G2" t="n">
-        <v>1584171996.317703</v>
+        <v>1338078347.1281</v>
       </c>
       <c r="H2" t="n">
-        <v>225.1470932343341</v>
+        <v>60.50425213733803</v>
       </c>
       <c r="I2" t="n">
-        <v>680.8324096253896</v>
+        <v>214.6277029303527</v>
       </c>
       <c r="J2" t="n">
-        <v>1338078347.1281</v>
+        <v>265565018.2470056</v>
       </c>
       <c r="K2" t="n">
-        <v>60.50425213733803</v>
+        <v>6.667193842428753</v>
       </c>
       <c r="L2" t="n">
-        <v>214.6277029303527</v>
+        <v>23.08270275014829</v>
       </c>
       <c r="M2" t="n">
-        <v>265565018.2470056</v>
-      </c>
-      <c r="N2" t="n">
-        <v>6.667193842428753</v>
-      </c>
-      <c r="O2" t="n">
-        <v>23.08270275014829</v>
-      </c>
-      <c r="P2" t="n">
         <v>6139583.068739802</v>
       </c>
     </row>
@@ -1132,48 +1075,39 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>604.5821272263487</v>
+        <v>481.5656708036506</v>
       </c>
       <c r="C3" t="n">
-        <v>780.8938728493939</v>
+        <v>764.7066101312035</v>
       </c>
       <c r="D3" t="n">
-        <v>881765226.632076</v>
+        <v>1687667188.817399</v>
       </c>
       <c r="E3" t="n">
-        <v>372.7813106039199</v>
+        <v>181.68636368164</v>
       </c>
       <c r="F3" t="n">
-        <v>750.9423203341649</v>
+        <v>499.3838888145954</v>
       </c>
       <c r="G3" t="n">
-        <v>816167004.876194</v>
+        <v>719741466.3429611</v>
       </c>
       <c r="H3" t="n">
-        <v>181.68636368164</v>
+        <v>49.64595776882005</v>
       </c>
       <c r="I3" t="n">
-        <v>499.3838888145954</v>
+        <v>153.4161094240039</v>
       </c>
       <c r="J3" t="n">
-        <v>719741466.3429611</v>
+        <v>135687961.8067113</v>
       </c>
       <c r="K3" t="n">
-        <v>49.64595776882005</v>
+        <v>4.620747572021741</v>
       </c>
       <c r="L3" t="n">
-        <v>153.4161094240039</v>
+        <v>14.70704859783348</v>
       </c>
       <c r="M3" t="n">
-        <v>135687961.8067113</v>
-      </c>
-      <c r="N3" t="n">
-        <v>4.620747572021741</v>
-      </c>
-      <c r="O3" t="n">
-        <v>14.70704859783348</v>
-      </c>
-      <c r="P3" t="n">
         <v>2492393.541350836</v>
       </c>
     </row>

</xml_diff>